<commit_message>
fix(investments): enhance CAS/Excel parser, ISIN matching, and market price guards
</commit_message>
<xml_diff>
--- a/parser-tests/fixtures/groww-portfolio.xlsx
+++ b/parser-tests/fixtures/groww-portfolio.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -420,6 +420,9 @@
       <c r="E3" t="str">
         <v>Invested Amount (INR)</v>
       </c>
+      <c r="F3" t="str">
+        <v>ISIN</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -437,6 +440,9 @@
       <c r="E4">
         <v>5025</v>
       </c>
+      <c r="F4" t="str">
+        <v>INF332K01RS0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -454,6 +460,9 @@
       <c r="E5">
         <v>45000</v>
       </c>
+      <c r="F5" t="str">
+        <v>INF179KC1000</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -471,10 +480,13 @@
       <c r="E6">
         <v>60000</v>
       </c>
+      <c r="F6" t="str">
+        <v>INF200K01VA0</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>